<commit_message>
refactor: adiciona csv bruto de pesagens e tratado
</commit_message>
<xml_diff>
--- a/Aula-02/pesagens-tratada.xlsx
+++ b/Aula-02/pesagens-tratada.xlsx
@@ -30,55 +30,127 @@
     <t>peso_t</t>
   </si>
   <si>
+    <t>coluna obs</t>
+  </si>
+  <si>
     <t>A</t>
   </si>
   <si>
     <t>T-03</t>
   </si>
   <si>
+    <t>Inconsistência- Data no padrão do Brasil</t>
+  </si>
+  <si>
+    <t>talhão 21</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e formato T-NN errado</t>
+  </si>
+  <si>
+    <t>a</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e letra minuscula</t>
+  </si>
+  <si>
     <t>T-21</t>
   </si>
   <si>
-    <t>Quantos problemas há de cada tipo (duplicidade, inconsistência e valor ausente)?</t>
+    <t>t15</t>
+  </si>
+  <si>
+    <t>Inconsistência- Data no padrão do Brasil e duplicidade</t>
   </si>
   <si>
     <t>T-15</t>
   </si>
   <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e peso ausente</t>
+  </si>
+  <si>
+    <t>B</t>
+  </si>
+  <si>
+    <t>T-07</t>
+  </si>
+  <si>
+    <t>(vazio)</t>
+  </si>
+  <si>
+    <t>Turno B</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e formato de turno errado</t>
+  </si>
+  <si>
+    <t>T03</t>
+  </si>
+  <si>
+    <t>29.0</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e peso fora do padrão</t>
+  </si>
+  <si>
+    <t>T-12</t>
+  </si>
+  <si>
+    <t>C</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e pesagem errada</t>
+  </si>
+  <si>
+    <t>30800 kg</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e peso em kg</t>
+  </si>
+  <si>
+    <t>a) Quantos problemas há de cada tipo (duplicidade, inconsistência e valor ausente)?</t>
+  </si>
+  <si>
+    <t>t-21</t>
+  </si>
+  <si>
     <t>Duplicidade: 6</t>
   </si>
   <si>
     <t>Inconsistências: 134</t>
   </si>
   <si>
+    <t>Correto</t>
+  </si>
+  <si>
     <t>Valor ausente: 9</t>
   </si>
   <si>
-    <t>Quantas linhas de dados tem o arquivo bruto e quantas tem a aba tratado?</t>
+    <t>2 Inconsistências- Data no padrão do Brasil e talhão ausente</t>
+  </si>
+  <si>
+    <t>b) Quantas linhas de dados tem o arquivo bruto e quantas tem a aba tratado?</t>
   </si>
   <si>
     <t>Arquivo bruto: 100 e arquivo tratado: 94</t>
   </si>
   <si>
-    <t>Quantas toneladas seriam contadas em dobro se as repetições não fossem removidas?</t>
-  </si>
-  <si>
-    <t>(vazio)</t>
-  </si>
-  <si>
-    <t>coluna obs</t>
-  </si>
-  <si>
-    <t>B</t>
-  </si>
-  <si>
-    <t>Qual é a soma da coluna peso_t da aba tratado, sem as linhas cujo obs fala de
+    <t>29.2</t>
+  </si>
+  <si>
+    <t>c) Quantas toneladas seriam contadas em dobro se as repetições não fossem removidas?</t>
+  </si>
+  <si>
+    <t>2 Inconsistências- Data no padrão do Brasil e pesagem no formato errado</t>
+  </si>
+  <si>
+    <t>T-7</t>
+  </si>
+  <si>
+    <t>d) Qual é a soma da coluna peso_t da aba tratado, sem as linhas cujo obs fala de
 peso? Quantos caminhões entram nessa soma?</t>
   </si>
   <si>
-    <t>T-07</t>
-  </si>
-  <si>
     <t>2.588,3 toneladas. 88 camimhões. Se aceitar o valor dos caminhões com mais de 45 toneladas e fazer uma diferença de quantas toneladas foram entregadas a mais, ficaria 3,201,3 toneladas com 90 caminhões e estaria levando 613 toneladas a mais.</t>
   </si>
   <si>
@@ -88,82 +160,10 @@
     <t>frase (pense em duplicidade e em valor zero).</t>
   </si>
   <si>
+    <t>32,9 t</t>
+  </si>
+  <si>
     <t>Sim. Algumas linhas parecem duplicidade por terem dados iguais, mas não são porque elas têm códigos diferentes, como as linhas 10 e 14. Ou nas linhas que tem o valor igual a 0 e parecem estar vazio, mas são uma contagem certa como as linhas 52 e 92</t>
-  </si>
-  <si>
-    <t>Inconsistência- Data no padrão do Brasil</t>
-  </si>
-  <si>
-    <t>talhão 21</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e formato T-NN errado</t>
-  </si>
-  <si>
-    <t>a</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e letra minuscula</t>
-  </si>
-  <si>
-    <t>T-12</t>
-  </si>
-  <si>
-    <t>C</t>
-  </si>
-  <si>
-    <t>t15</t>
-  </si>
-  <si>
-    <t>Inconsistência- Data no padrão do Brasil e duplicidade</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e peso ausente</t>
-  </si>
-  <si>
-    <t>Turno B</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e formato de turno errado</t>
-  </si>
-  <si>
-    <t>T03</t>
-  </si>
-  <si>
-    <t>29.0</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e peso fora do padrão</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e pesagem errada</t>
-  </si>
-  <si>
-    <t>30800 kg</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e peso em kg</t>
-  </si>
-  <si>
-    <t>t-21</t>
-  </si>
-  <si>
-    <t>Correto</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e talhão ausente</t>
-  </si>
-  <si>
-    <t>29.2</t>
-  </si>
-  <si>
-    <t>2 Inconsistências- Data no padrão do Brasil e pesagem no formato errado</t>
-  </si>
-  <si>
-    <t>T-7</t>
-  </si>
-  <si>
-    <t>32,9 t</t>
   </si>
   <si>
     <t>2 Inconsistências- Data no padrão do Brasil e pesagem errada e acima de 45t</t>
@@ -213,10 +213,10 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
   <numFmts count="9">
-    <numFmt numFmtId="164" formatCode="yyyy&quot;-&quot;mm&quot;-&quot;dd"/>
-    <numFmt numFmtId="165" formatCode="dd&quot;/&quot;mm&quot;/&quot;yy"/>
-    <numFmt numFmtId="166" formatCode="0.0"/>
-    <numFmt numFmtId="167" formatCode="d.m"/>
+    <numFmt numFmtId="164" formatCode="dd&quot;/&quot;mm&quot;/&quot;yy"/>
+    <numFmt numFmtId="165" formatCode="yyyy&quot;-&quot;mm&quot;-&quot;dd"/>
+    <numFmt numFmtId="166" formatCode="d.m"/>
+    <numFmt numFmtId="167" formatCode="0.0"/>
     <numFmt numFmtId="168" formatCode="dd/mm/yy"/>
     <numFmt numFmtId="169" formatCode="dd/mm/yyyy"/>
     <numFmt numFmtId="170" formatCode="yyyy-mm-dd"/>
@@ -284,7 +284,7 @@
     <xf borderId="0" fillId="0" fontId="1" numFmtId="172" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
-    <xf borderId="0" fillId="0" fontId="1" numFmtId="164" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
+    <xf borderId="0" fillId="0" fontId="1" numFmtId="165" xfId="0" applyAlignment="1" applyFont="1" applyNumberFormat="1">
       <alignment readingOrder="0"/>
     </xf>
   </cellXfs>
@@ -532,364 +532,364 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>17</v>
+        <v>5</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1">
         <v>1001.0</v>
       </c>
-      <c r="B2" s="3">
+      <c r="B2" s="2">
         <v>46300.0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1">
         <v>28.4</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" s="1">
         <v>1002.0</v>
       </c>
-      <c r="B3" s="3">
+      <c r="B3" s="2">
         <v>46300.0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="E3" s="1">
         <v>30.9</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1">
         <v>1003.0</v>
       </c>
-      <c r="B4" s="3">
+      <c r="B4" s="2">
         <v>46300.0</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="1">
         <v>32.6</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1">
         <v>1004.0</v>
       </c>
-      <c r="B5" s="3">
+      <c r="B5" s="2">
         <v>46300.0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E5" s="5">
+        <v>13</v>
+      </c>
+      <c r="E5" s="4">
         <v>46233.0</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="1">
         <v>1005.0</v>
       </c>
-      <c r="B6" s="3">
+      <c r="B6" s="2">
         <v>46300.0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>32</v>
+        <v>14</v>
       </c>
       <c r="E6" s="1">
         <v>31.9</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1">
         <v>1006.0</v>
       </c>
-      <c r="B7" s="3">
+      <c r="B7" s="2">
         <v>46300.0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E7" s="1">
         <v>32.3</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="1">
         <v>1006.0</v>
       </c>
-      <c r="B8" s="3">
+      <c r="B8" s="2">
         <v>46300.0</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E8" s="1">
         <v>32.3</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="1">
         <v>1007.0</v>
       </c>
-      <c r="B9" s="3">
+      <c r="B9" s="2">
         <v>46300.0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
         <v>1008.0</v>
       </c>
-      <c r="B10" s="3">
+      <c r="B10" s="2">
         <v>46300.0</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="1">
         <v>29.6</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1">
         <v>1009.0</v>
       </c>
-      <c r="B11" s="3">
+      <c r="B11" s="2">
         <v>46300.0</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>35</v>
+        <v>21</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" s="1">
         <v>30.6</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>36</v>
+        <v>22</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="1">
         <v>1010.0</v>
       </c>
-      <c r="B12" s="3">
+      <c r="B12" s="2">
         <v>46300.0</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>37</v>
+        <v>23</v>
       </c>
       <c r="E12" s="1">
         <v>28.2</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1">
         <v>1011.0</v>
       </c>
-      <c r="B13" s="3">
+      <c r="B13" s="2">
         <v>46300.0</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" s="1">
         <v>29.4</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1">
         <v>1012.0</v>
       </c>
-      <c r="B14" s="3">
+      <c r="B14" s="2">
         <v>46300.0</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E14" s="1">
         <v>29.6</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1">
         <v>1013.0</v>
       </c>
-      <c r="B15" s="3">
+      <c r="B15" s="2">
         <v>46300.0</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E15" s="1" t="s">
-        <v>38</v>
+        <v>24</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="1">
         <v>1014.0</v>
       </c>
-      <c r="B16" s="3">
+      <c r="B16" s="2">
         <v>46300.0</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E16" s="1">
         <v>33.3</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="1">
         <v>1015.0</v>
       </c>
-      <c r="B17" s="3">
+      <c r="B17" s="2">
         <v>46300.0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E17" s="1">
         <v>32.0</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="1">
         <v>1016.0</v>
       </c>
-      <c r="B18" s="3">
+      <c r="B18" s="2">
         <v>46300.0</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E18" s="1" t="s">
-        <v>41</v>
+        <v>29</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="1">
         <v>1017.0</v>
       </c>
-      <c r="B19" s="3">
+      <c r="B19" s="2">
         <v>46300.0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E19" s="1">
         <v>30.2</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="20">
@@ -900,16 +900,16 @@
         <v>46300.0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E20" s="1">
         <v>28.2</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="21">
@@ -920,16 +920,16 @@
         <v>46300.0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E21" s="1">
         <v>27.1</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="22">
@@ -940,16 +940,16 @@
         <v>46301.0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="E22" s="1">
         <v>28.3</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="23">
@@ -960,16 +960,16 @@
         <v>46301.0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E23" s="1">
         <v>28.7</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="24">
@@ -980,13 +980,13 @@
         <v>46301.0</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="E24" s="1">
         <v>26.7</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>45</v>
+        <v>37</v>
       </c>
     </row>
     <row r="25">
@@ -997,16 +997,16 @@
         <v>46301.0</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E25" s="1">
         <v>30.2</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="26">
@@ -1017,16 +1017,16 @@
         <v>46301.0</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E26" s="1" t="s">
-        <v>46</v>
+        <v>40</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
     </row>
     <row r="27">
@@ -1037,16 +1037,16 @@
         <v>46301.0</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="E27" s="1">
         <v>32.6</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="28">
@@ -1057,16 +1057,16 @@
         <v>46301.0</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E28" s="1">
         <v>32.9</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="29">
@@ -1080,10 +1080,10 @@
         <v>18</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="30">
@@ -1097,13 +1097,13 @@
         <v>18</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E30" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="31">
@@ -1117,13 +1117,13 @@
         <v>18</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E31" s="1">
         <v>29.8</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="32">
@@ -1137,7 +1137,7 @@
         <v>18</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" s="1">
         <v>303.0</v>
@@ -1157,13 +1157,13 @@
         <v>51</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E33" s="1">
         <v>32.1</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>29</v>
+        <v>12</v>
       </c>
     </row>
     <row r="34">
@@ -1177,13 +1177,13 @@
         <v>18</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E34" s="1">
         <v>32.7</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
@@ -1197,13 +1197,13 @@
         <v>18</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E35" s="1">
         <v>31.4</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="36">
@@ -1217,13 +1217,13 @@
         <v>18</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E36" s="1">
         <v>31.4</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>33</v>
+        <v>15</v>
       </c>
     </row>
     <row r="37">
@@ -1234,16 +1234,16 @@
         <v>46301.0</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E37" s="1">
         <v>29.5</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="38">
@@ -1254,16 +1254,16 @@
         <v>46301.0</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E38" s="1">
         <v>32.6</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="39">
@@ -1274,7 +1274,7 @@
         <v>46301.0</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E39" s="1">
         <v>30.7</v>
@@ -1291,16 +1291,16 @@
         <v>46301.0</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E40" s="1">
         <v>31.0</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="41">
@@ -1311,16 +1311,16 @@
         <v>46301.0</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>26</v>
+        <v>9</v>
       </c>
       <c r="E41" s="1">
         <v>27.9</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="42">
@@ -1331,16 +1331,16 @@
         <v>46302.0</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E42" s="1">
         <v>31.0</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="43">
@@ -1351,16 +1351,16 @@
         <v>46302.0</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E43" s="1">
         <v>30.1</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="44">
@@ -1371,13 +1371,13 @@
         <v>46302.0</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="45">
@@ -1388,16 +1388,16 @@
         <v>46302.0</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E45" s="1">
         <v>29.2</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="46">
@@ -1408,16 +1408,16 @@
         <v>46302.0</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E46" s="1">
         <v>32.2</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="47">
@@ -1428,7 +1428,7 @@
         <v>46302.0</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D47" s="1" t="s">
         <v>53</v>
@@ -1437,7 +1437,7 @@
         <v>26.2</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>27</v>
+        <v>10</v>
       </c>
     </row>
     <row r="48">
@@ -1448,16 +1448,16 @@
         <v>46302.0</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E48" s="1">
         <v>33.2</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="49">
@@ -1471,13 +1471,13 @@
         <v>18</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E49" s="1" t="s">
         <v>54</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>42</v>
+        <v>30</v>
       </c>
     </row>
     <row r="50">
@@ -1491,13 +1491,13 @@
         <v>18</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E50" s="1">
         <v>32.9</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="51">
@@ -1511,13 +1511,13 @@
         <v>18</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E51" s="1">
         <v>31.2</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="52">
@@ -1531,13 +1531,13 @@
         <v>18</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E52" s="1">
         <v>0.0</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="53">
@@ -1551,13 +1551,13 @@
         <v>18</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E53" s="1" t="s">
         <v>55</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>39</v>
+        <v>25</v>
       </c>
     </row>
     <row r="54">
@@ -1588,13 +1588,13 @@
         <v>18</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E55" s="1">
         <v>32.2</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="56">
@@ -1605,16 +1605,16 @@
         <v>46302.0</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E56" s="1">
         <v>29.4</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="57">
@@ -1625,16 +1625,16 @@
         <v>46302.0</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E57" s="1">
         <v>29.3</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="58">
@@ -1645,16 +1645,16 @@
         <v>46302.0</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E58" s="1">
         <v>27.9</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="59">
@@ -1665,16 +1665,16 @@
         <v>46302.0</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E59" s="1">
         <v>33.3</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="60">
@@ -1685,16 +1685,16 @@
         <v>46302.0</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E60" s="1">
         <v>33.1</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="61">
@@ -1705,16 +1705,16 @@
         <v>46303.0</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E61" s="1">
         <v>32.8</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="62">
@@ -1725,16 +1725,16 @@
         <v>46303.0</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E62" s="1">
         <v>26.7</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="63">
@@ -1745,16 +1745,16 @@
         <v>46303.0</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E63" s="1">
         <v>27.1</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="64">
@@ -1765,16 +1765,16 @@
         <v>46303.0</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E64" s="1">
         <v>26.7</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="65">
@@ -1785,16 +1785,16 @@
         <v>46303.0</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E65" s="1">
         <v>30.4</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="66">
@@ -1805,16 +1805,16 @@
         <v>46303.0</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
         <v>30.6</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="67">
@@ -1825,13 +1825,13 @@
         <v>46303.0</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D67" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>34</v>
+        <v>17</v>
       </c>
     </row>
     <row r="68">
@@ -1845,13 +1845,13 @@
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E68" s="1">
         <v>26.3</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="69">
@@ -1865,13 +1865,13 @@
         <v>18</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E69" s="1">
         <v>33.2</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="70">
@@ -1885,13 +1885,13 @@
         <v>18</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E70" s="1">
         <v>27.2</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="71">
@@ -1905,7 +1905,7 @@
         <v>18</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E71" s="1">
         <v>310.0</v>
@@ -1925,13 +1925,13 @@
         <v>18</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E72" s="1">
         <v>31.8</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="73">
@@ -1945,13 +1945,13 @@
         <v>18</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E73" s="1">
         <v>31.2</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="74">
@@ -1962,7 +1962,7 @@
         <v>46303.0</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E74" s="1">
         <v>30.1</v>
@@ -1979,16 +1979,16 @@
         <v>46303.0</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E75" s="1">
         <v>30.0</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="76">
@@ -1999,16 +1999,16 @@
         <v>46303.0</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E76" s="1">
         <v>32.6</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
@@ -2019,16 +2019,16 @@
         <v>46303.0</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E77" s="1">
         <v>28.2</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="78">
@@ -2039,10 +2039,10 @@
         <v>46303.0</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E78" s="1">
         <v>31.0</v>
@@ -2059,16 +2059,16 @@
         <v>46303.0</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E79" s="1">
         <v>31.9</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="80">
@@ -2079,16 +2079,16 @@
         <v>46304.0</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E80" s="1">
         <v>28.3</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="81">
@@ -2099,16 +2099,16 @@
         <v>46304.0</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E81" s="1">
         <v>28.9</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="82">
@@ -2119,16 +2119,16 @@
         <v>46304.0</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E82" s="1">
         <v>29.9</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>44</v>
+        <v>35</v>
       </c>
     </row>
     <row r="83">
@@ -2139,16 +2139,16 @@
         <v>46304.0</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E83" s="1">
         <v>28.8</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="84">
@@ -2159,16 +2159,16 @@
         <v>46304.0</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E84" s="1">
         <v>28.9</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85">
@@ -2179,16 +2179,16 @@
         <v>46304.0</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E85" s="1">
         <v>26.4</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="86">
@@ -2199,16 +2199,16 @@
         <v>46304.0</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E86" s="1">
         <v>30.8</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="87">
@@ -2222,13 +2222,13 @@
         <v>18</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E87" s="1">
         <v>26.2</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
@@ -2242,13 +2242,13 @@
         <v>18</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E88" s="1">
         <v>28.5</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
@@ -2262,13 +2262,13 @@
         <v>18</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E89" s="1">
         <v>29.4</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="90">
@@ -2282,13 +2282,13 @@
         <v>18</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E90" s="1">
         <v>29.7</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="91">
@@ -2302,13 +2302,13 @@
         <v>18</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E91" s="1">
         <v>30.3</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="92">
@@ -2322,13 +2322,13 @@
         <v>18</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E92" s="1">
         <v>0.0</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="93">
@@ -2356,16 +2356,16 @@
         <v>46304.0</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E94" s="1">
         <v>30.2</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="95">
@@ -2376,16 +2376,16 @@
         <v>46304.0</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E95" s="1" t="s">
         <v>59</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>40</v>
+        <v>28</v>
       </c>
     </row>
     <row r="96">
@@ -2396,16 +2396,16 @@
         <v>46304.0</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E96" s="1">
         <v>30.1</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="97">
@@ -2416,16 +2416,16 @@
         <v>46304.0</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E97" s="1">
         <v>27.5</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>25</v>
+        <v>8</v>
       </c>
     </row>
     <row r="98">
@@ -2439,7 +2439,7 @@
         <v>18</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E98" s="1">
         <v>31.2</v>
@@ -2459,7 +2459,7 @@
         <v>18</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E99" s="1">
         <v>26.3</v>
@@ -2496,7 +2496,7 @@
         <v>46304.0</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>28</v>
+        <v>11</v>
       </c>
       <c r="D101" s="1" t="s">
         <v>62</v>
@@ -2541,14 +2541,14 @@
       <c r="A2" s="1">
         <v>1001.0</v>
       </c>
-      <c r="B2" s="2">
+      <c r="B2" s="3">
         <v>46300.0</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E2" s="1">
         <v>28.4</v>
@@ -2559,14 +2559,14 @@
       <c r="A3" s="1">
         <v>1002.0</v>
       </c>
-      <c r="B3" s="2">
+      <c r="B3" s="3">
         <v>46300.0</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1">
         <v>30.9</v>
@@ -2576,14 +2576,14 @@
       <c r="A4" s="1">
         <v>1003.0</v>
       </c>
-      <c r="B4" s="2">
+      <c r="B4" s="3">
         <v>46300.0</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E4" s="1">
         <v>32.6</v>
@@ -2593,14 +2593,14 @@
       <c r="A5" s="1">
         <v>1004.0</v>
       </c>
-      <c r="B5" s="2">
+      <c r="B5" s="3">
         <v>46300.0</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E5" s="1">
         <v>30.7</v>
@@ -2610,14 +2610,14 @@
       <c r="A6" s="1">
         <v>1005.0</v>
       </c>
-      <c r="B6" s="2">
+      <c r="B6" s="3">
         <v>46300.0</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E6" s="1">
         <v>31.9</v>
@@ -2627,51 +2627,51 @@
       <c r="A7" s="1">
         <v>1006.0</v>
       </c>
-      <c r="B7" s="2">
+      <c r="B7" s="3">
         <v>46300.0</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E7" s="1">
         <v>32.3</v>
       </c>
     </row>
     <row r="8">
-      <c r="B8" s="2"/>
+      <c r="B8" s="3"/>
     </row>
     <row r="9">
       <c r="A9" s="1">
         <v>1007.0</v>
       </c>
-      <c r="B9" s="2">
+      <c r="B9" s="3">
         <v>46300.0</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E9" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="1">
         <v>1008.0</v>
       </c>
-      <c r="B10" s="2">
+      <c r="B10" s="3">
         <v>46300.0</v>
       </c>
       <c r="C10" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E10" s="1">
         <v>29.6</v>
@@ -2681,14 +2681,14 @@
       <c r="A11" s="1">
         <v>1009.0</v>
       </c>
-      <c r="B11" s="2">
+      <c r="B11" s="3">
         <v>46300.0</v>
       </c>
       <c r="C11" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E11" s="1">
         <v>30.6</v>
@@ -2698,14 +2698,14 @@
       <c r="A12" s="1">
         <v>1010.0</v>
       </c>
-      <c r="B12" s="2">
+      <c r="B12" s="3">
         <v>46300.0</v>
       </c>
       <c r="C12" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E12" s="1">
         <v>28.2</v>
@@ -2715,14 +2715,14 @@
       <c r="A13" s="1">
         <v>1011.0</v>
       </c>
-      <c r="B13" s="2">
+      <c r="B13" s="3">
         <v>46300.0</v>
       </c>
       <c r="C13" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E13" s="1">
         <v>29.4</v>
@@ -2732,14 +2732,14 @@
       <c r="A14" s="1">
         <v>1012.0</v>
       </c>
-      <c r="B14" s="2">
+      <c r="B14" s="3">
         <v>46300.0</v>
       </c>
       <c r="C14" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E14" s="1">
         <v>29.6</v>
@@ -2749,16 +2749,16 @@
       <c r="A15" s="1">
         <v>1013.0</v>
       </c>
-      <c r="B15" s="2">
+      <c r="B15" s="3">
         <v>46300.0</v>
       </c>
       <c r="C15" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="E15" s="4">
+        <v>19</v>
+      </c>
+      <c r="E15" s="5">
         <v>29.0</v>
       </c>
     </row>
@@ -2766,14 +2766,14 @@
       <c r="A16" s="1">
         <v>1014.0</v>
       </c>
-      <c r="B16" s="2">
+      <c r="B16" s="3">
         <v>46300.0</v>
       </c>
       <c r="C16" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E16" s="1">
         <v>33.3</v>
@@ -2783,16 +2783,16 @@
       <c r="A17" s="1">
         <v>1015.0</v>
       </c>
-      <c r="B17" s="2">
+      <c r="B17" s="3">
         <v>46300.0</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E17" s="4">
+        <v>26</v>
+      </c>
+      <c r="E17" s="5">
         <v>32.0</v>
       </c>
     </row>
@@ -2800,14 +2800,14 @@
       <c r="A18" s="1">
         <v>1016.0</v>
       </c>
-      <c r="B18" s="2">
+      <c r="B18" s="3">
         <v>46300.0</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E18" s="1">
         <v>30.8</v>
@@ -2817,14 +2817,14 @@
       <c r="A19" s="1">
         <v>1017.0</v>
       </c>
-      <c r="B19" s="2">
+      <c r="B19" s="3">
         <v>46300.0</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D19" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E19" s="1">
         <v>30.2</v>
@@ -2834,14 +2834,14 @@
       <c r="A20" s="1">
         <v>1018.0</v>
       </c>
-      <c r="B20" s="2">
+      <c r="B20" s="3">
         <v>46300.0</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E20" s="1">
         <v>28.2</v>
@@ -2851,14 +2851,14 @@
       <c r="A21" s="1">
         <v>1019.0</v>
       </c>
-      <c r="B21" s="2">
+      <c r="B21" s="3">
         <v>46300.0</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E21" s="1">
         <v>27.1</v>
@@ -2868,14 +2868,14 @@
       <c r="A22" s="1">
         <v>1020.0</v>
       </c>
-      <c r="B22" s="2">
+      <c r="B22" s="3">
         <v>46301.0</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E22" s="1">
         <v>28.3</v>
@@ -2885,14 +2885,14 @@
       <c r="A23" s="1">
         <v>1021.0</v>
       </c>
-      <c r="B23" s="2">
+      <c r="B23" s="3">
         <v>46301.0</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E23" s="1">
         <v>28.7</v>
@@ -2902,14 +2902,14 @@
       <c r="A24" s="1">
         <v>1022.0</v>
       </c>
-      <c r="B24" s="2">
+      <c r="B24" s="3">
         <v>46301.0</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E24" s="1">
         <v>26.7</v>
@@ -2919,14 +2919,14 @@
       <c r="A25" s="1">
         <v>1023.0</v>
       </c>
-      <c r="B25" s="2">
+      <c r="B25" s="3">
         <v>46301.0</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E25" s="1">
         <v>30.2</v>
@@ -2936,14 +2936,14 @@
       <c r="A26" s="1">
         <v>1024.0</v>
       </c>
-      <c r="B26" s="2">
+      <c r="B26" s="3">
         <v>46301.0</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E26" s="1">
         <v>29.2</v>
@@ -2953,14 +2953,14 @@
       <c r="A27" s="1">
         <v>1025.0</v>
       </c>
-      <c r="B27" s="2">
+      <c r="B27" s="3">
         <v>46301.0</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E27" s="1">
         <v>32.6</v>
@@ -2970,14 +2970,14 @@
       <c r="A28" s="1">
         <v>1026.0</v>
       </c>
-      <c r="B28" s="2">
+      <c r="B28" s="3">
         <v>46301.0</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E28" s="1">
         <v>32.9</v>
@@ -2987,31 +2987,31 @@
       <c r="A29" s="1">
         <v>1027.0</v>
       </c>
-      <c r="B29" s="2">
+      <c r="B29" s="3">
         <v>46301.0</v>
       </c>
       <c r="C29" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E29" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="1">
         <v>1028.0</v>
       </c>
-      <c r="B30" s="2">
+      <c r="B30" s="3">
         <v>46301.0</v>
       </c>
       <c r="C30" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E30" s="1">
         <v>32.9</v>
@@ -3021,14 +3021,14 @@
       <c r="A31" s="1">
         <v>1029.0</v>
       </c>
-      <c r="B31" s="2">
+      <c r="B31" s="3">
         <v>46301.0</v>
       </c>
       <c r="C31" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E31" s="1">
         <v>29.8</v>
@@ -3038,14 +3038,14 @@
       <c r="A32" s="1">
         <v>1030.0</v>
       </c>
-      <c r="B32" s="2">
+      <c r="B32" s="3">
         <v>46301.0</v>
       </c>
       <c r="C32" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E32" s="1">
         <v>30.3</v>
@@ -3055,14 +3055,14 @@
       <c r="A33" s="1">
         <v>1031.0</v>
       </c>
-      <c r="B33" s="2">
+      <c r="B33" s="3">
         <v>46301.0</v>
       </c>
       <c r="C33" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E33" s="1">
         <v>32.1</v>
@@ -3072,14 +3072,14 @@
       <c r="A34" s="1">
         <v>1032.0</v>
       </c>
-      <c r="B34" s="2">
+      <c r="B34" s="3">
         <v>46301.0</v>
       </c>
       <c r="C34" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E34" s="1">
         <v>32.7</v>
@@ -3089,34 +3089,34 @@
       <c r="A35" s="1">
         <v>1033.0</v>
       </c>
-      <c r="B35" s="2">
+      <c r="B35" s="3">
         <v>46301.0</v>
       </c>
       <c r="C35" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E35" s="1">
         <v>31.4</v>
       </c>
     </row>
     <row r="36">
-      <c r="B36" s="2"/>
+      <c r="B36" s="3"/>
     </row>
     <row r="37">
       <c r="A37" s="1">
         <v>1034.0</v>
       </c>
-      <c r="B37" s="2">
+      <c r="B37" s="3">
         <v>46301.0</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E37" s="1">
         <v>29.5</v>
@@ -3126,14 +3126,14 @@
       <c r="A38" s="1">
         <v>1035.0</v>
       </c>
-      <c r="B38" s="2">
+      <c r="B38" s="3">
         <v>46301.0</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E38" s="1">
         <v>32.6</v>
@@ -3143,14 +3143,14 @@
       <c r="A39" s="1">
         <v>1036.0</v>
       </c>
-      <c r="B39" s="2">
+      <c r="B39" s="3">
         <v>46301.0</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E39" s="1">
         <v>30.7</v>
@@ -3160,16 +3160,16 @@
       <c r="A40" s="1">
         <v>1037.0</v>
       </c>
-      <c r="B40" s="2">
+      <c r="B40" s="3">
         <v>46301.0</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E40" s="4">
+        <v>16</v>
+      </c>
+      <c r="E40" s="5">
         <v>31.0</v>
       </c>
     </row>
@@ -3177,14 +3177,14 @@
       <c r="A41" s="1">
         <v>1038.0</v>
       </c>
-      <c r="B41" s="2">
+      <c r="B41" s="3">
         <v>46301.0</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E41" s="1">
         <v>27.9</v>
@@ -3194,16 +3194,16 @@
       <c r="A42" s="1">
         <v>1039.0</v>
       </c>
-      <c r="B42" s="2">
+      <c r="B42" s="3">
         <v>46302.0</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D42" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E42" s="4">
+        <v>16</v>
+      </c>
+      <c r="E42" s="5">
         <v>31.0</v>
       </c>
     </row>
@@ -3211,14 +3211,14 @@
       <c r="A43" s="1">
         <v>1040.0</v>
       </c>
-      <c r="B43" s="2">
+      <c r="B43" s="3">
         <v>46302.0</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D43" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E43" s="1">
         <v>30.1</v>
@@ -3228,31 +3228,31 @@
       <c r="A44" s="1">
         <v>1041.0</v>
       </c>
-      <c r="B44" s="2">
+      <c r="B44" s="3">
         <v>46302.0</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D44" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="1">
         <v>1042.0</v>
       </c>
-      <c r="B45" s="2">
+      <c r="B45" s="3">
         <v>46302.0</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D45" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E45" s="1">
         <v>29.2</v>
@@ -3262,14 +3262,14 @@
       <c r="A46" s="1">
         <v>1043.0</v>
       </c>
-      <c r="B46" s="2">
+      <c r="B46" s="3">
         <v>46302.0</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E46" s="1">
         <v>32.2</v>
@@ -3279,14 +3279,14 @@
       <c r="A47" s="1">
         <v>1044.0</v>
       </c>
-      <c r="B47" s="2">
+      <c r="B47" s="3">
         <v>46302.0</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E47" s="1">
         <v>26.2</v>
@@ -3296,14 +3296,14 @@
       <c r="A48" s="1">
         <v>1045.0</v>
       </c>
-      <c r="B48" s="2">
+      <c r="B48" s="3">
         <v>46302.0</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D48" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E48" s="1">
         <v>33.2</v>
@@ -3313,16 +3313,16 @@
       <c r="A49" s="1">
         <v>1046.0</v>
       </c>
-      <c r="B49" s="2">
+      <c r="B49" s="3">
         <v>46302.0</v>
       </c>
       <c r="C49" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="E49" s="4">
+        <v>13</v>
+      </c>
+      <c r="E49" s="5">
         <v>33.0</v>
       </c>
     </row>
@@ -3330,14 +3330,14 @@
       <c r="A50" s="1">
         <v>1047.0</v>
       </c>
-      <c r="B50" s="2">
+      <c r="B50" s="3">
         <v>46302.0</v>
       </c>
       <c r="C50" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E50" s="1">
         <v>32.9</v>
@@ -3347,14 +3347,14 @@
       <c r="A51" s="1">
         <v>1048.0</v>
       </c>
-      <c r="B51" s="2">
+      <c r="B51" s="3">
         <v>46302.0</v>
       </c>
       <c r="C51" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E51" s="1">
         <v>31.2</v>
@@ -3364,14 +3364,14 @@
       <c r="A52" s="1">
         <v>1049.0</v>
       </c>
-      <c r="B52" s="2">
+      <c r="B52" s="3">
         <v>46302.0</v>
       </c>
       <c r="C52" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E52" s="1">
         <v>0.0</v>
@@ -3381,14 +3381,14 @@
       <c r="A53" s="1">
         <v>1050.0</v>
       </c>
-      <c r="B53" s="2">
+      <c r="B53" s="3">
         <v>46302.0</v>
       </c>
       <c r="C53" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E53" s="1">
         <v>32.1</v>
@@ -3398,16 +3398,16 @@
       <c r="A54" s="1">
         <v>1051.0</v>
       </c>
-      <c r="B54" s="2">
+      <c r="B54" s="3">
         <v>46302.0</v>
       </c>
       <c r="C54" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="E54" s="4">
+        <v>20</v>
+      </c>
+      <c r="E54" s="5">
         <v>31.0</v>
       </c>
     </row>
@@ -3415,14 +3415,14 @@
       <c r="A55" s="1">
         <v>1052.0</v>
       </c>
-      <c r="B55" s="2">
+      <c r="B55" s="3">
         <v>46302.0</v>
       </c>
       <c r="C55" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E55" s="1">
         <v>32.2</v>
@@ -3432,14 +3432,14 @@
       <c r="A56" s="1">
         <v>1053.0</v>
       </c>
-      <c r="B56" s="2">
+      <c r="B56" s="3">
         <v>46302.0</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E56" s="1">
         <v>29.4</v>
@@ -3449,14 +3449,14 @@
       <c r="A57" s="1">
         <v>1054.0</v>
       </c>
-      <c r="B57" s="2">
+      <c r="B57" s="3">
         <v>46302.0</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E57" s="1">
         <v>29.3</v>
@@ -3466,14 +3466,14 @@
       <c r="A58" s="1">
         <v>1055.0</v>
       </c>
-      <c r="B58" s="2">
+      <c r="B58" s="3">
         <v>46302.0</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E58" s="1">
         <v>27.9</v>
@@ -3483,14 +3483,14 @@
       <c r="A59" s="1">
         <v>1056.0</v>
       </c>
-      <c r="B59" s="2">
+      <c r="B59" s="3">
         <v>46302.0</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E59" s="1">
         <v>33.3</v>
@@ -3500,14 +3500,14 @@
       <c r="A60" s="1">
         <v>1057.0</v>
       </c>
-      <c r="B60" s="2">
+      <c r="B60" s="3">
         <v>46302.0</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E60" s="1">
         <v>33.1</v>
@@ -3517,14 +3517,14 @@
       <c r="A61" s="1">
         <v>1058.0</v>
       </c>
-      <c r="B61" s="2">
+      <c r="B61" s="3">
         <v>46303.0</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E61" s="1">
         <v>32.8</v>
@@ -3534,14 +3534,14 @@
       <c r="A62" s="1">
         <v>1059.0</v>
       </c>
-      <c r="B62" s="2">
+      <c r="B62" s="3">
         <v>46303.0</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D62" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E62" s="1">
         <v>26.7</v>
@@ -3551,14 +3551,14 @@
       <c r="A63" s="1">
         <v>1060.0</v>
       </c>
-      <c r="B63" s="2">
+      <c r="B63" s="3">
         <v>46303.0</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E63" s="1">
         <v>27.1</v>
@@ -3568,14 +3568,14 @@
       <c r="A64" s="1">
         <v>1061.0</v>
       </c>
-      <c r="B64" s="2">
+      <c r="B64" s="3">
         <v>46303.0</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E64" s="1">
         <v>26.7</v>
@@ -3585,14 +3585,14 @@
       <c r="A65" s="1">
         <v>1062.0</v>
       </c>
-      <c r="B65" s="2">
+      <c r="B65" s="3">
         <v>46303.0</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E65" s="1">
         <v>30.4</v>
@@ -3602,14 +3602,14 @@
       <c r="A66" s="1">
         <v>1063.0</v>
       </c>
-      <c r="B66" s="2">
+      <c r="B66" s="3">
         <v>46303.0</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E66" s="1">
         <v>30.6</v>
@@ -3619,31 +3619,31 @@
       <c r="A67" s="1">
         <v>1064.0</v>
       </c>
-      <c r="B67" s="2">
+      <c r="B67" s="3">
         <v>46303.0</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D67" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="E67" s="1" t="s">
         <v>20</v>
-      </c>
-      <c r="E67" s="1" t="s">
-        <v>16</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="1">
         <v>1065.0</v>
       </c>
-      <c r="B68" s="2">
+      <c r="B68" s="3">
         <v>46303.0</v>
       </c>
       <c r="C68" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E68" s="1">
         <v>26.3</v>
@@ -3653,14 +3653,14 @@
       <c r="A69" s="1">
         <v>1066.0</v>
       </c>
-      <c r="B69" s="2">
+      <c r="B69" s="3">
         <v>46303.0</v>
       </c>
       <c r="C69" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E69" s="1">
         <v>33.2</v>
@@ -3670,14 +3670,14 @@
       <c r="A70" s="1">
         <v>1067.0</v>
       </c>
-      <c r="B70" s="2">
+      <c r="B70" s="3">
         <v>46303.0</v>
       </c>
       <c r="C70" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D70" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E70" s="1">
         <v>27.2</v>
@@ -3687,16 +3687,16 @@
       <c r="A71" s="1">
         <v>1068.0</v>
       </c>
-      <c r="B71" s="2">
+      <c r="B71" s="3">
         <v>46303.0</v>
       </c>
       <c r="C71" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D71" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="E71" s="4">
+        <v>26</v>
+      </c>
+      <c r="E71" s="5">
         <v>31.0</v>
       </c>
     </row>
@@ -3704,14 +3704,14 @@
       <c r="A72" s="1">
         <v>1069.0</v>
       </c>
-      <c r="B72" s="2">
+      <c r="B72" s="3">
         <v>46303.0</v>
       </c>
       <c r="C72" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D72" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E72" s="1">
         <v>31.8</v>
@@ -3721,14 +3721,14 @@
       <c r="A73" s="1">
         <v>1070.0</v>
       </c>
-      <c r="B73" s="2">
+      <c r="B73" s="3">
         <v>46303.0</v>
       </c>
       <c r="C73" s="1" t="s">
         <v>18</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E73" s="1">
         <v>31.2</v>
@@ -3738,14 +3738,14 @@
       <c r="A74" s="1">
         <v>1071.0</v>
       </c>
-      <c r="B74" s="2">
+      <c r="B74" s="3">
         <v>46303.0</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E74" s="1">
         <v>30.1</v>
@@ -3755,16 +3755,16 @@
       <c r="A75" s="1">
         <v>1072.0</v>
       </c>
-      <c r="B75" s="2">
+      <c r="B75" s="3">
         <v>46303.0</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D75" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="E75" s="4">
+        <v>16</v>
+      </c>
+      <c r="E75" s="5">
         <v>30.0</v>
       </c>
     </row>
@@ -3772,14 +3772,14 @@
       <c r="A76" s="1">
         <v>1073.0</v>
       </c>
-      <c r="B76" s="2">
+      <c r="B76" s="3">
         <v>46303.0</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D76" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E76" s="1">
         <v>32.6</v>
@@ -3789,14 +3789,14 @@
       <c r="A77" s="1">
         <v>1074.0</v>
       </c>
-      <c r="B77" s="2">
+      <c r="B77" s="3">
         <v>46303.0</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E77" s="1">
         <v>28.2</v>
@@ -3806,14 +3806,14 @@
       <c r="A78" s="1">
         <v>1075.0</v>
       </c>
-      <c r="B78" s="2">
+      <c r="B78" s="3">
         <v>46303.0</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E78" s="10">
         <v>30.0</v>
@@ -3823,14 +3823,14 @@
       <c r="A79" s="1">
         <v>1076.0</v>
       </c>
-      <c r="B79" s="2">
+      <c r="B79" s="3">
         <v>46303.0</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E79" s="1">
         <v>31.9</v>
@@ -3840,14 +3840,14 @@
       <c r="A80" s="1">
         <v>1077.0</v>
       </c>
-      <c r="B80" s="2">
+      <c r="B80" s="3">
         <v>46304.0</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E80" s="1">
         <v>28.3</v>
@@ -3857,14 +3857,14 @@
       <c r="A81" s="1">
         <v>1078.0</v>
       </c>
-      <c r="B81" s="2">
+      <c r="B81" s="3">
         <v>46304.0</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E81" s="1">
         <v>28.9</v>
@@ -3878,10 +3878,10 @@
         <v>46304.0</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E82" s="1">
         <v>29.9</v>
@@ -3895,10 +3895,10 @@
         <v>46304.0</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E83" s="1">
         <v>28.8</v>
@@ -3912,10 +3912,10 @@
         <v>46304.0</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E84" s="1">
         <v>28.9</v>
@@ -3929,10 +3929,10 @@
         <v>46304.0</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E85" s="1">
         <v>26.4</v>
@@ -3946,10 +3946,10 @@
         <v>46304.0</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E86" s="1">
         <v>30.8</v>
@@ -3966,7 +3966,7 @@
         <v>18</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E87" s="1">
         <v>26.2</v>
@@ -3983,7 +3983,7 @@
         <v>18</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E88" s="1">
         <v>28.5</v>
@@ -4000,7 +4000,7 @@
         <v>18</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E89" s="1">
         <v>29.4</v>
@@ -4017,7 +4017,7 @@
         <v>18</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E90" s="1">
         <v>29.7</v>
@@ -4034,7 +4034,7 @@
         <v>18</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="E91" s="1">
         <v>30.3</v>
@@ -4051,7 +4051,7 @@
         <v>18</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="E92" s="1">
         <v>0.0</v>
@@ -4068,7 +4068,7 @@
         <v>18</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>16</v>
+        <v>20</v>
       </c>
       <c r="E93" s="1">
         <v>27.6</v>
@@ -4082,10 +4082,10 @@
         <v>46304.0</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="E94" s="1">
         <v>30.2</v>
@@ -4099,10 +4099,10 @@
         <v>46304.0</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E95" s="1">
         <v>27.7</v>
@@ -4116,10 +4116,10 @@
         <v>46304.0</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E96" s="1">
         <v>30.1</v>
@@ -4133,10 +4133,10 @@
         <v>46304.0</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>31</v>
+        <v>27</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="E97" s="1">
         <v>27.5</v>
@@ -4171,33 +4171,33 @@
   <sheetData>
     <row r="1">
       <c r="A1" s="1" t="s">
-        <v>8</v>
+        <v>31</v>
       </c>
     </row>
     <row r="2">
       <c r="A2" s="1" t="s">
-        <v>10</v>
+        <v>33</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>11</v>
+        <v>34</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>12</v>
+        <v>36</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" s="1" t="s">
-        <v>13</v>
+        <v>38</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="1" t="s">
-        <v>14</v>
+        <v>39</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="1" t="s">
-        <v>15</v>
+        <v>41</v>
       </c>
     </row>
     <row r="8">
@@ -4207,27 +4207,27 @@
     </row>
     <row r="10">
       <c r="A10" s="1" t="s">
-        <v>19</v>
+        <v>44</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="1" t="s">
-        <v>21</v>
+        <v>45</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="1" t="s">
-        <v>22</v>
+        <v>46</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="1" t="s">
-        <v>23</v>
+        <v>47</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="1" t="s">
-        <v>24</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>

</xml_diff>